<commit_message>
Correciones e inclusiones de datos faltantes al análisis (incompleto)
</commit_message>
<xml_diff>
--- a/backend/test-files/Staff-Time-Summary-Report-prueba (2).xlsx
+++ b/backend/test-files/Staff-Time-Summary-Report-prueba (2).xlsx
@@ -349,7 +349,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
-    <numFmt numFmtId="1621" formatCode="##,###,##0.00##"/>
+    <numFmt numFmtId="171" formatCode="##,###,##0.00##"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -384,6 +384,13 @@
     <font>
       <b val="0"/>
       <i val="0"/>
+      <sz val="9.75"/>
+      <color theme="1"/>
+      <name val="Verdana"/>
+    </font>
+    <font>
+      <b val="0"/>
+      <i val="0"/>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Verdana"/>
@@ -400,13 +407,6 @@
       <i val="0"/>
       <sz val="8"/>
       <color rgb="FFD3D3D3"/>
-      <name val="Verdana"/>
-    </font>
-    <font>
-      <b val="0"/>
-      <i val="0"/>
-      <sz val="9.75"/>
-      <color theme="1"/>
       <name val="Verdana"/>
     </font>
   </fonts>
@@ -452,28 +452,28 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="right" vertical="top" readingOrder="1" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="1621" fontId="3" fillId="0" borderId="0" xfId="0">
+    <xf numFmtId="171" fontId="3" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="right" vertical="top" readingOrder="1" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="1621" fontId="7" fillId="0" borderId="0" xfId="0">
+    <xf numFmtId="171" fontId="4" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0">
-      <alignment horizontal="left" vertical="top" readingOrder="1" wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="left" vertical="top" readingOrder="1" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0">
-      <alignment horizontal="right" vertical="top" readingOrder="1" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="1621" fontId="5" fillId="0" borderId="0" xfId="0">
-      <alignment horizontal="right" vertical="top" readingOrder="1" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0">
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="left" vertical="top" readingOrder="1" wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0">
+      <alignment horizontal="right" vertical="top" readingOrder="1" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="6" fillId="0" borderId="0" xfId="0">
+      <alignment horizontal="right" vertical="top" readingOrder="1" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0">
+      <alignment horizontal="left" vertical="top" readingOrder="1" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="center" vertical="top" readingOrder="1" wrapText="1" shrinkToFit="1"/>
     </xf>
   </cellXfs>
@@ -3683,7 +3683,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{D2EF9E9E-F22E-4A69-92AF-28B3F731F261}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{C7AD65DC-6A66-4611-AC52-8E1F333435AB}" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>

</xml_diff>